<commit_message>
add id name to test
</commit_message>
<xml_diff>
--- a/linkage/data_processing_elements_linkage-FRA.xlsx
+++ b/linkage/data_processing_elements_linkage-FRA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/292c22834a0ab190/Documents/ProPASS/Linkage/FIREA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="216" documentId="8_{2907C675-FC1E-45BC-80C8-03193858AA4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3462D897-4A04-4FD0-B780-10ABE05EDEF5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{026C1775-36E5-45DE-AAA9-46F3F15F496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="79">
   <si>
     <t>index</t>
   </si>
@@ -156,9 +156,6 @@
   </si>
   <si>
     <t>adm_id</t>
-  </si>
-  <si>
-    <t>TBD</t>
   </si>
   <si>
     <t>ICD10 codes for the causes of death are present in the database in the most detailed format (e.g., C169)</t>
@@ -300,6 +297,12 @@
   </si>
   <si>
     <t>format(kuolpv, "%m")</t>
+  </si>
+  <si>
+    <t>id_creation</t>
+  </si>
+  <si>
+    <t>id_var</t>
   </si>
 </sst>
 </file>
@@ -432,12 +435,8 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -754,7 +753,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}">
   <dimension ref="A1:S15"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" style="5" customWidth="1"/>
@@ -842,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>38</v>
@@ -854,26 +853,30 @@
         <v>18</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>39</v>
+        <v>57</v>
+      </c>
+      <c r="G2" t="s">
+        <v>78</v>
       </c>
       <c r="P2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q2" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="Q2" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="R2" s="11"/>
-      <c r="S2" s="6"/>
+      <c r="R2" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="S2" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>19</v>
@@ -885,25 +888,25 @@
         <v>18</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
@@ -911,7 +914,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>21</v>
@@ -923,25 +926,25 @@
         <v>18</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R4" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="S4" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -949,7 +952,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>23</v>
@@ -961,25 +964,25 @@
         <v>18</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="Q5" s="5" t="s">
-        <v>42</v>
-      </c>
       <c r="R5" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -987,37 +990,37 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="P6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q6" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="Q6" s="5" t="s">
-        <v>42</v>
-      </c>
       <c r="R6" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="105" x14ac:dyDescent="0.25">
@@ -1025,10 +1028,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>30</v>
@@ -1037,31 +1040,31 @@
         <v>18</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H7" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="P7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M7" s="9" t="s">
+      <c r="Q7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="R7" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="S7" s="9" t="s">
         <v>65</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q7" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="R7" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="S7" s="9" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:19" ht="60" x14ac:dyDescent="0.25">
@@ -1069,10 +1072,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>31</v>
@@ -1081,28 +1084,28 @@
         <v>18</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M8" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q8" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S8" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="60" x14ac:dyDescent="0.25">
@@ -1110,10 +1113,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>32</v>
@@ -1122,28 +1125,28 @@
         <v>18</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M9" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="P9" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q9" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R9" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S9" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="60" x14ac:dyDescent="0.25">
@@ -1151,7 +1154,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>25</v>
@@ -1163,28 +1166,28 @@
         <v>18</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M10" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="P10" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q10" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S10" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="60" x14ac:dyDescent="0.25">
@@ -1192,10 +1195,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>34</v>
@@ -1204,28 +1207,28 @@
         <v>18</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H11" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M11" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M11" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="P11" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q11" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R11" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S11" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:19" ht="75" x14ac:dyDescent="0.25">
@@ -1233,10 +1236,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>35</v>
@@ -1245,31 +1248,31 @@
         <v>18</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H12" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M12" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="N12" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="P12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M12" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="N12" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="P12" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q12" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R12" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S12" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="75" x14ac:dyDescent="0.25">
@@ -1277,10 +1280,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>36</v>
@@ -1289,28 +1292,28 @@
         <v>18</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M13" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P13" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M13" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="P13" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q13" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R13" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S13" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="90" x14ac:dyDescent="0.25">
@@ -1318,10 +1321,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>37</v>
@@ -1330,28 +1333,28 @@
         <v>18</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H14" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M14" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P14" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="M14" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="P14" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="Q14" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R14" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S14" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:19" ht="150" x14ac:dyDescent="0.25">
@@ -1359,7 +1362,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>26</v>
@@ -1371,28 +1374,28 @@
         <v>18</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="P15" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="Q15" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changed id name to id1
</commit_message>
<xml_diff>
--- a/linkage/data_processing_elements_linkage-FRA.xlsx
+++ b/linkage/data_processing_elements_linkage-FRA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/292c22834a0ab190/Documents/ProPASS/Linkage/FIREA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{026C1775-36E5-45DE-AAA9-46F3F15F496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{026C1775-36E5-45DE-AAA9-46F3F15F496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ECA05DE-9E88-4FDD-BF87-479CDF98E220}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
+    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15840" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -302,7 +302,7 @@
     <t>id_creation</t>
   </si>
   <si>
-    <t>id_var</t>
+    <t>id1</t>
   </si>
 </sst>
 </file>
@@ -436,7 +436,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -753,7 +753,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}">
   <dimension ref="A1:S15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" style="5" customWidth="1"/>

</xml_diff>

<commit_message>
correct day and month algorithm
</commit_message>
<xml_diff>
--- a/linkage/data_processing_elements_linkage-FRA.xlsx
+++ b/linkage/data_processing_elements_linkage-FRA.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/292c22834a0ab190/Documents/ProPASS/Linkage/FIREA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{026C1775-36E5-45DE-AAA9-46F3F15F496B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ECA05DE-9E88-4FDD-BF87-479CDF98E220}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6286E3C8-BB77-4980-98B3-F462086E01D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-90" windowWidth="29040" windowHeight="15840" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{63444C23-9E00-4348-B1ED-05F831BC47B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$S$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Feuil1!$A$1:$R$15</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="75">
   <si>
     <t>index</t>
   </si>
@@ -77,9 +77,6 @@
     <t>input_keywords</t>
   </si>
   <si>
-    <t>internal_comment</t>
-  </si>
-  <si>
     <t>Mlstr_harmo::comment</t>
   </si>
   <si>
@@ -182,9 +179,6 @@
     <t>case_when</t>
   </si>
   <si>
-    <t>ZC: Changed "^J010" to "^J10"; duplicate value of "^J17" was changed to "^J16".</t>
-  </si>
-  <si>
     <t>dth_heart_dis_nhanes</t>
   </si>
   <si>
@@ -204,12 +198,6 @@
   </si>
   <si>
     <t>dth_injuries_acc_nhanes</t>
-  </si>
-  <si>
-    <t>ZC: Changed "^J010" to "^J10"; added missing code "^J16"; removed whitespace since it was interfering with pattern detection.</t>
-  </si>
-  <si>
-    <t>ZC: To account for missing codes, changed rules to case_when and added condition to code as missing instead of "No" - note that this condition requires missing ICD-10 codes to be coded as NA in the input data. Same comment for all cause of death variables below.</t>
   </si>
   <si>
     <t>dataset_FRA</t>
@@ -357,18 +345,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -400,9 +382,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -415,7 +394,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -436,7 +418,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -752,8 +734,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}">
-  <dimension ref="A1:S15"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" style="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" style="5" customWidth="1"/>
@@ -767,17 +749,16 @@
     <col min="10" max="10" width="21" style="5" customWidth="1"/>
     <col min="11" max="11" width="27.5703125" style="5" customWidth="1"/>
     <col min="12" max="12" width="17.5703125" style="5" customWidth="1"/>
-    <col min="13" max="13" width="27.85546875" style="7" customWidth="1"/>
-    <col min="14" max="14" width="36.5703125" style="7" customWidth="1"/>
-    <col min="15" max="15" width="24.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="12.85546875" style="5" customWidth="1"/>
-    <col min="17" max="17" width="18.85546875" style="5" customWidth="1"/>
-    <col min="18" max="18" width="14.5703125" style="5" customWidth="1"/>
-    <col min="19" max="19" width="57.42578125" style="5" customWidth="1"/>
-    <col min="20" max="16384" width="11.5703125" style="5"/>
+    <col min="13" max="13" width="27.85546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="24.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.85546875" style="5" customWidth="1"/>
+    <col min="16" max="16" width="18.85546875" style="5" customWidth="1"/>
+    <col min="17" max="17" width="14.5703125" style="5" customWidth="1"/>
+    <col min="18" max="18" width="57.42578125" style="5" customWidth="1"/>
+    <col min="19" max="16384" width="11.5703125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="4" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" s="4" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -788,7 +769,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -817,10 +798,10 @@
       <c r="M1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>13</v>
       </c>
       <c r="P1" s="3" t="s">
@@ -832,574 +813,562 @@
       <c r="R1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
-      </c>
-      <c r="P2" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="O2" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="Q2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="R2" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="S2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="Q2" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="R2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="M3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>62</v>
+      <c r="O3" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="M4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>62</v>
+      <c r="O4" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="S4" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="E5" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G5" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>63</v>
+        <v>53</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="P5" s="5" t="s">
         <v>40</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="S5" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>64</v>
+      <c r="M6" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="P6" s="5" t="s">
         <v>40</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="S6" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="105" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>48</v>
+        <v>54</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P7" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R7" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="H7" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q7" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R7" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S7" s="9" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>49</v>
+        <v>54</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M8" s="9" t="s">
-        <v>64</v>
-      </c>
       <c r="P8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q8" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R8" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S8" s="9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="Q8" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>50</v>
+        <v>54</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O9" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="9" t="s">
-        <v>64</v>
-      </c>
       <c r="P9" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R9" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S9" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="Q9" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R9" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>9</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G10" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M10" s="9" t="s">
+      <c r="P10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q10" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R10" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="P10" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q10" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R10" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S10" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>49</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="7" t="s">
+      <c r="H11" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O11" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M11" s="9" t="s">
-        <v>64</v>
-      </c>
       <c r="P11" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q11" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R11" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S11" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="Q11" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R11" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G12" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12" s="7" t="s">
+      <c r="H12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M12" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="N12" s="9" t="s">
-        <v>47</v>
-      </c>
       <c r="P12" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q12" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R12" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S12" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" ht="75" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="Q12" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R12" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F13" s="5" t="s">
+      <c r="G13" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H13" s="7" t="s">
+      <c r="H13" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M13" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M13" s="9" t="s">
-        <v>64</v>
-      </c>
       <c r="P13" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q13" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R13" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S13" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" ht="90" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="Q13" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R13" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="90" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="10" t="s">
         <v>54</v>
       </c>
+      <c r="C14" s="9" t="s">
+        <v>52</v>
+      </c>
       <c r="D14" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="M14" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="M14" s="9" t="s">
-        <v>64</v>
-      </c>
       <c r="P14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q14" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R14" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S14" s="9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" ht="150" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+      <c r="Q14" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R14" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="E15" s="5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M15" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="N15" s="9" t="s">
-        <v>55</v>
+      <c r="M15" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="P15" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="Q15" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R15" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="S15" s="9" t="s">
-        <v>73</v>
+        <v>41</v>
+      </c>
+      <c r="Q15" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="R15" s="8" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S15" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}"/>
+  <autoFilter ref="A1:R15" xr:uid="{2A96D0D0-036F-4639-8FBF-4A4CEF797E7C}"/>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>